<commit_message>
Quito opocion para ejecutar cargar pto
</commit_message>
<xml_diff>
--- a/archivos/tabla_variedades.xlsx
+++ b/archivos/tabla_variedades.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESTADISTICA\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE3970BF-0BBB-4C82-8B96-A8F154ACE420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{969D51BC-FF0F-4EBF-A690-459F569BA160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-735" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1290" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tabla_variedades" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tabla_variedades!$A$1:$H$1356</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tabla_variedades!$A$1:$H$1366</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5315" uniqueCount="1424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5319" uniqueCount="1426">
   <si>
     <t>id</t>
   </si>
@@ -4295,6 +4295,12 @@
   </si>
   <si>
     <t>2007</t>
+  </si>
+  <si>
+    <t>2422</t>
+  </si>
+  <si>
+    <t>DAMASCUS_</t>
   </si>
 </sst>
 </file>
@@ -5147,7 +5153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1366"/>
+  <dimension ref="A1:H1367"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="11.42578125" style="1"/>
@@ -6135,7 +6141,7 @@
         <v>2049</v>
       </c>
       <c r="G38">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -6811,7 +6817,7 @@
         <v>2341</v>
       </c>
       <c r="G64">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H64">
         <v>1</v>
@@ -8293,7 +8299,7 @@
         <v>2299</v>
       </c>
       <c r="G121">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H121">
         <v>1</v>
@@ -8943,7 +8949,7 @@
         <v>2264</v>
       </c>
       <c r="G146">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H146" t="s">
         <v>11</v>
@@ -16951,7 +16957,7 @@
         <v>5941</v>
       </c>
       <c r="G454">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H454" t="s">
         <v>11</v>
@@ -24543,7 +24549,7 @@
         <v>0</v>
       </c>
       <c r="G746">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H746" t="s">
         <v>11</v>
@@ -28313,7 +28319,7 @@
         <v>0</v>
       </c>
       <c r="G891">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H891" t="s">
         <v>11</v>
@@ -29546,7 +29552,7 @@
         <v>938</v>
       </c>
       <c r="B939" t="s">
-        <v>950</v>
+        <v>1425</v>
       </c>
       <c r="C939" t="s">
         <v>9</v>
@@ -33539,7 +33545,7 @@
         <v>0</v>
       </c>
       <c r="G1092">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H1092" t="s">
         <v>11</v>
@@ -39051,7 +39057,7 @@
         <v>2430</v>
       </c>
       <c r="G1304">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H1304">
         <v>1</v>
@@ -39103,7 +39109,7 @@
         <v>2424</v>
       </c>
       <c r="G1306">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H1306">
         <v>1</v>
@@ -39207,7 +39213,7 @@
         <v>2426</v>
       </c>
       <c r="G1310">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H1310">
         <v>1</v>
@@ -40400,10 +40406,10 @@
         <v>2440</v>
       </c>
       <c r="G1356">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H1356">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1357" spans="1:8" x14ac:dyDescent="0.25">
@@ -40423,10 +40429,10 @@
         <v>1413</v>
       </c>
       <c r="G1357">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H1357">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1358" spans="1:8" x14ac:dyDescent="0.25">
@@ -40446,10 +40452,10 @@
         <v>1414</v>
       </c>
       <c r="G1358">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H1358">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1359" spans="1:8" x14ac:dyDescent="0.25">
@@ -40469,10 +40475,10 @@
         <v>1415</v>
       </c>
       <c r="G1359">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H1359">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1360" spans="1:8" x14ac:dyDescent="0.25">
@@ -40492,10 +40498,10 @@
         <v>1416</v>
       </c>
       <c r="G1360">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H1360">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1361" spans="2:8" x14ac:dyDescent="0.25">
@@ -40515,10 +40521,10 @@
         <v>1417</v>
       </c>
       <c r="G1361">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H1361">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1362" spans="2:8" x14ac:dyDescent="0.25">
@@ -40538,10 +40544,10 @@
         <v>1418</v>
       </c>
       <c r="G1362">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H1362">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1363" spans="2:8" x14ac:dyDescent="0.25">
@@ -40561,10 +40567,10 @@
         <v>1419</v>
       </c>
       <c r="G1363">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H1363">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1364" spans="2:8" x14ac:dyDescent="0.25">
@@ -40584,10 +40590,10 @@
         <v>1420</v>
       </c>
       <c r="G1364">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H1364">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1365" spans="2:8" x14ac:dyDescent="0.25">
@@ -40607,10 +40613,10 @@
         <v>1421</v>
       </c>
       <c r="G1365">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H1365">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1366" spans="2:8" x14ac:dyDescent="0.25">
@@ -40630,14 +40636,37 @@
         <v>1423</v>
       </c>
       <c r="G1366">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H1366">
-        <v>0</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1367" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1367" t="s">
+        <v>950</v>
+      </c>
+      <c r="C1367" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1367" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1367">
+        <v>26</v>
+      </c>
+      <c r="F1367" s="1" t="s">
+        <v>1424</v>
+      </c>
+      <c r="G1367">
+        <v>1</v>
+      </c>
+      <c r="H1367">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1356" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H1366" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
actualiza bautizos y aplicaciones
</commit_message>
<xml_diff>
--- a/archivos/tabla_variedades.xlsx
+++ b/archivos/tabla_variedades.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESTADISTICA\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{969D51BC-FF0F-4EBF-A690-459F569BA160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0E35C2-4E98-4DC7-B5A6-FA0ABB7E2F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1290" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tabla_variedades" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tabla_variedades!$A$1:$H$1366</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tabla_variedades!$A$1:$H$1374</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5319" uniqueCount="1426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5347" uniqueCount="1434">
   <si>
     <t>id</t>
   </si>
@@ -4301,6 +4301,30 @@
   </si>
   <si>
     <t>DAMASCUS_</t>
+  </si>
+  <si>
+    <t>MOONPHASE</t>
+  </si>
+  <si>
+    <t>ORANGE PARTY</t>
+  </si>
+  <si>
+    <t>PROGRESS</t>
+  </si>
+  <si>
+    <t>BLUEBERRY</t>
+  </si>
+  <si>
+    <t>TIGER</t>
+  </si>
+  <si>
+    <t>MISS FRANCE</t>
+  </si>
+  <si>
+    <t>CREME CARAMEL</t>
+  </si>
+  <si>
+    <t>0</t>
   </si>
 </sst>
 </file>
@@ -5153,7 +5177,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1367"/>
+  <dimension ref="A1:H1374"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="11.42578125" style="1"/>
@@ -8943,7 +8967,7 @@
         <v>17</v>
       </c>
       <c r="E146">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F146">
         <v>2264</v>
@@ -24543,7 +24567,7 @@
         <v>17</v>
       </c>
       <c r="E746">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F746">
         <v>0</v>
@@ -39213,7 +39237,7 @@
         <v>2426</v>
       </c>
       <c r="G1310">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H1310">
         <v>1</v>
@@ -40665,8 +40689,169 @@
         <v>1</v>
       </c>
     </row>
+    <row r="1368" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1368" t="s">
+        <v>1426</v>
+      </c>
+      <c r="C1368" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1368" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1368">
+        <v>0</v>
+      </c>
+      <c r="F1368" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="G1368">
+        <v>8</v>
+      </c>
+      <c r="H1368">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1369" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1369" t="s">
+        <v>1427</v>
+      </c>
+      <c r="C1369" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1369" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1369">
+        <v>0</v>
+      </c>
+      <c r="F1369" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="G1369">
+        <v>8</v>
+      </c>
+      <c r="H1369">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1370" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1370" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C1370" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1370" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1370">
+        <v>0</v>
+      </c>
+      <c r="F1370" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="G1370">
+        <v>8</v>
+      </c>
+      <c r="H1370">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1371" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1371" t="s">
+        <v>1429</v>
+      </c>
+      <c r="C1371" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1371" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1371">
+        <v>0</v>
+      </c>
+      <c r="F1371" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="G1371">
+        <v>8</v>
+      </c>
+      <c r="H1371">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1372" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1372" t="s">
+        <v>1430</v>
+      </c>
+      <c r="C1372" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1372" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1372">
+        <v>0</v>
+      </c>
+      <c r="F1372" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="G1372">
+        <v>8</v>
+      </c>
+      <c r="H1372">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1373" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1373" t="s">
+        <v>1431</v>
+      </c>
+      <c r="C1373" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1373" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1373">
+        <v>0</v>
+      </c>
+      <c r="F1373" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="G1373">
+        <v>8</v>
+      </c>
+      <c r="H1373">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1374" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1374" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C1374" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1374" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1374">
+        <v>0</v>
+      </c>
+      <c r="F1374" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="G1374">
+        <v>8</v>
+      </c>
+      <c r="H1374">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H1366" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H1374" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>

</xml_diff>